<commit_message>
補正 5 筆覆核後 Ticker 空白的公司（Apple、Boeing、Corpay、American Express、Autoliv）
</commit_message>
<xml_diff>
--- a/news_daily/2026-08-30.xlsx
+++ b/news_daily/2026-08-30.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="完整新聞" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="主要負面事件" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="待人工覆核" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="待補分析" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="執行紀錄" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整新聞" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主要負面事件" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待人工覆核" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待補分析" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="執行紀錄" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'完整新聞'!$A$1:$BL$12</definedName>
@@ -27,16 +27,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -61,7 +58,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -69,21 +66,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1055,7 +1044,11 @@
           <t>US</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Apple Inc.</t>
@@ -1215,7 +1208,7 @@
       <c r="BH3" s="3" t="inlineStr"/>
       <c r="BI3" s="3" t="inlineStr">
         <is>
-          <t>Event_Code|Level|事件中文</t>
+          <t>Event_Code|Level|Ticker|事件中文</t>
         </is>
       </c>
       <c r="BJ3" s="3" t="inlineStr"/>
@@ -3394,7 +3387,11 @@
           <t>US</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Apple Inc.</t>
@@ -3554,7 +3551,7 @@
       <c r="BH2" s="3" t="inlineStr"/>
       <c r="BI2" s="3" t="inlineStr">
         <is>
-          <t>Event_Code|Level|事件中文</t>
+          <t>Event_Code|Level|Ticker|事件中文</t>
         </is>
       </c>
       <c r="BJ2" s="3" t="inlineStr"/>

</xml_diff>